<commit_message>
More one time usign it
</commit_message>
<xml_diff>
--- a/core/src/main/resources/baseFiles/excel/Reports.xlsx
+++ b/core/src/main/resources/baseFiles/excel/Reports.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="217">
   <si>
     <t>Firm</t>
   </si>
@@ -39,172 +39,646 @@
     <t>Lawyers Registered</t>
   </si>
   <si>
-    <t>Cassels</t>
+    <t>Lee &amp; Ko</t>
+  </si>
+  <si>
+    <t>04min 00s</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>TAN Law</t>
+  </si>
+  <si>
+    <t>Balter, Guth, Aloni &amp; Co</t>
+  </si>
+  <si>
+    <t>Tanner DeWitt</t>
+  </si>
+  <si>
+    <t>03min 52s</t>
+  </si>
+  <si>
+    <t>Gadens</t>
+  </si>
+  <si>
+    <t>03min 36s</t>
+  </si>
+  <si>
+    <t>Yuen Law</t>
+  </si>
+  <si>
+    <t>03min 07s</t>
+  </si>
+  <si>
+    <t>Lipa Meir &amp; Co</t>
+  </si>
+  <si>
+    <t>03min 04s</t>
+  </si>
+  <si>
+    <t>TA Law</t>
+  </si>
+  <si>
+    <t>02min 55s</t>
+  </si>
+  <si>
+    <t>LHAG</t>
+  </si>
+  <si>
+    <t>02min 33s</t>
+  </si>
+  <si>
+    <t>Wrays</t>
+  </si>
+  <si>
+    <t>02min 31s</t>
+  </si>
+  <si>
+    <t>Shoob &amp; Co</t>
+  </si>
+  <si>
+    <t>02min 30s</t>
+  </si>
+  <si>
+    <t>Saga Legal</t>
+  </si>
+  <si>
+    <t>Remfry &amp; Sagar</t>
+  </si>
+  <si>
+    <t>02min 21s</t>
+  </si>
+  <si>
+    <t>Aquinas Law Alliance</t>
+  </si>
+  <si>
+    <t>01min 54s</t>
+  </si>
+  <si>
+    <t>YKVN</t>
+  </si>
+  <si>
+    <t>01min 33s</t>
+  </si>
+  <si>
+    <t>Frasers</t>
+  </si>
+  <si>
+    <t>01min 21s</t>
+  </si>
+  <si>
+    <t>Domnern Somgiat &amp; Boonma</t>
+  </si>
+  <si>
+    <t>01min 18s</t>
+  </si>
+  <si>
+    <t>Kim Chang &amp; Lee</t>
+  </si>
+  <si>
+    <t>01min 15s</t>
+  </si>
+  <si>
+    <t>Wong Partnership</t>
+  </si>
+  <si>
+    <t>01min 11s</t>
+  </si>
+  <si>
+    <t>Mohanadass Partnership</t>
+  </si>
+  <si>
+    <t>01min 08s</t>
+  </si>
+  <si>
+    <t>Harry Elias</t>
+  </si>
+  <si>
+    <t>01min 05s</t>
+  </si>
+  <si>
+    <t>RIAA Barker Gillette</t>
+  </si>
+  <si>
+    <t>01min 02s</t>
+  </si>
+  <si>
+    <t>Axis Law Chambers</t>
+  </si>
+  <si>
+    <t>FGE Ebrahim Hosain</t>
+  </si>
+  <si>
+    <t>01min 00s</t>
+  </si>
+  <si>
+    <t>SG &amp; Co Lawyers</t>
+  </si>
+  <si>
+    <t>59s</t>
+  </si>
+  <si>
+    <t>Sayat Zholshy &amp; Partners</t>
+  </si>
+  <si>
+    <t>Boase Cohen &amp; Collins</t>
+  </si>
+  <si>
+    <t>58s</t>
+  </si>
+  <si>
+    <t>Desai &amp; Diwanji</t>
+  </si>
+  <si>
+    <t>57s</t>
+  </si>
+  <si>
+    <t>LS Horizon</t>
+  </si>
+  <si>
+    <t>56s</t>
+  </si>
+  <si>
+    <t>ALMT Legal</t>
+  </si>
+  <si>
+    <t>55s</t>
+  </si>
+  <si>
+    <t>JTJB International Lawyers</t>
+  </si>
+  <si>
+    <t>54s</t>
+  </si>
+  <si>
+    <t>Yoon &amp; Yang</t>
+  </si>
+  <si>
+    <t>48s</t>
+  </si>
+  <si>
+    <t>SIGNUM</t>
+  </si>
+  <si>
+    <t>46s</t>
+  </si>
+  <si>
+    <t>Kochhar &amp; Co</t>
+  </si>
+  <si>
+    <t>45s</t>
+  </si>
+  <si>
+    <t>Al Alawi &amp; Co</t>
+  </si>
+  <si>
+    <t>Bun &amp; Associates</t>
+  </si>
+  <si>
+    <t>44s</t>
+  </si>
+  <si>
+    <t>Shardul Amarchand Mangaldas &amp; Co</t>
+  </si>
+  <si>
+    <t>43s</t>
+  </si>
+  <si>
+    <t>VILAF</t>
+  </si>
+  <si>
+    <t>38s</t>
+  </si>
+  <si>
+    <t>Asia Liuh IP</t>
+  </si>
+  <si>
+    <t>37s</t>
+  </si>
+  <si>
+    <t>Rajani Associates</t>
+  </si>
+  <si>
+    <t>36s</t>
+  </si>
+  <si>
+    <t>Dhir &amp; Dhir</t>
+  </si>
+  <si>
+    <t>35s</t>
+  </si>
+  <si>
+    <t>H-F &amp; Co</t>
+  </si>
+  <si>
+    <t>34s</t>
+  </si>
+  <si>
+    <t>S&amp;O IP</t>
+  </si>
+  <si>
+    <t>32s</t>
+  </si>
+  <si>
+    <t>LAW Partnership</t>
+  </si>
+  <si>
+    <t>D. L. And F. De Saram</t>
+  </si>
+  <si>
+    <t>31s</t>
+  </si>
+  <si>
+    <t>Haidermota &amp; Co</t>
+  </si>
+  <si>
+    <t>30s</t>
+  </si>
+  <si>
+    <t>Fox And Mandal</t>
+  </si>
+  <si>
+    <t>Stratage Law</t>
+  </si>
+  <si>
+    <t>Bowers</t>
+  </si>
+  <si>
+    <t>29s</t>
+  </si>
+  <si>
+    <t>Zhongzi Law</t>
+  </si>
+  <si>
+    <t>Ramdas &amp; Wong</t>
+  </si>
+  <si>
+    <t>28s</t>
+  </si>
+  <si>
+    <t>S Horowitz &amp; Co</t>
+  </si>
+  <si>
+    <t>Zan Hub</t>
+  </si>
+  <si>
+    <t>SIP Law</t>
+  </si>
+  <si>
+    <t>26s</t>
+  </si>
+  <si>
+    <t>Dhaval Vussonji &amp; Associates</t>
+  </si>
+  <si>
+    <t>Eldan Law</t>
+  </si>
+  <si>
+    <t>Manuela António</t>
+  </si>
+  <si>
+    <t>25s</t>
+  </si>
+  <si>
+    <t>Vision &amp; Associates</t>
+  </si>
+  <si>
+    <t>Bross And Partners</t>
+  </si>
+  <si>
+    <t>24s</t>
+  </si>
+  <si>
+    <t>RCL Chambers Law</t>
+  </si>
+  <si>
+    <t>Gross &amp; Co</t>
+  </si>
+  <si>
+    <t>Cornelius Lane &amp; Mufti</t>
+  </si>
+  <si>
+    <t>23s</t>
+  </si>
+  <si>
+    <t>Deacons</t>
+  </si>
+  <si>
+    <t>22s</t>
+  </si>
+  <si>
+    <t>Vanguard Lawyers Tokyo</t>
+  </si>
+  <si>
+    <t>Nurmansyah &amp; Muzdalifah</t>
+  </si>
+  <si>
+    <t>Makes &amp; Partners Law</t>
+  </si>
+  <si>
+    <t>21s</t>
+  </si>
+  <si>
+    <t>SGLA Law</t>
+  </si>
+  <si>
+    <t>FCLaw</t>
+  </si>
+  <si>
+    <t>20s</t>
+  </si>
+  <si>
+    <t>ABS And Co</t>
+  </si>
+  <si>
+    <t>Bhandari Naqvi Riaz</t>
+  </si>
+  <si>
+    <t>YYC Legal</t>
+  </si>
+  <si>
+    <t>M&amp;D LAW</t>
+  </si>
+  <si>
+    <t>19s</t>
+  </si>
+  <si>
+    <t>Sierra Legal</t>
+  </si>
+  <si>
+    <t>Mohsin Tayebaly &amp; Co</t>
+  </si>
+  <si>
+    <t>18s</t>
+  </si>
+  <si>
+    <t>Russell McVeagh</t>
+  </si>
+  <si>
+    <t>MBIP</t>
+  </si>
+  <si>
+    <t>Tian Yuan</t>
+  </si>
+  <si>
+    <t>17s</t>
+  </si>
+  <si>
+    <t>GKC Partners</t>
+  </si>
+  <si>
+    <t>Barnea And Co</t>
+  </si>
+  <si>
+    <t>16s</t>
+  </si>
+  <si>
+    <t>Helmsman</t>
+  </si>
+  <si>
+    <t>15s</t>
+  </si>
+  <si>
+    <t>Global Vietnam Lawyers</t>
+  </si>
+  <si>
+    <t>Chadha &amp; Co</t>
+  </si>
+  <si>
+    <t>DSKLegal</t>
+  </si>
+  <si>
+    <t>Baohua Law</t>
+  </si>
+  <si>
+    <t>Doogue + George</t>
+  </si>
+  <si>
+    <t>Moroğlu Arseven</t>
+  </si>
+  <si>
+    <t>14s</t>
+  </si>
+  <si>
+    <t>HY Leung &amp; Co</t>
+  </si>
+  <si>
+    <t>Beijing East IP</t>
+  </si>
+  <si>
+    <t>13s</t>
+  </si>
+  <si>
+    <t>Tommy Thomas</t>
+  </si>
+  <si>
+    <t>Al Busaidy, Mansoor Jamal &amp; Co</t>
+  </si>
+  <si>
+    <t>Deheheng Law</t>
+  </si>
+  <si>
+    <t>Hugill &amp; Ip</t>
+  </si>
+  <si>
+    <t>Hiways</t>
+  </si>
+  <si>
+    <t>12s</t>
+  </si>
+  <si>
+    <t>Malley And Co</t>
+  </si>
+  <si>
+    <t>Maheshwari &amp; Co</t>
+  </si>
+  <si>
+    <t>11s</t>
+  </si>
+  <si>
+    <t>Collyer Law</t>
+  </si>
+  <si>
+    <t>Lektou</t>
+  </si>
+  <si>
+    <t>Tiruchelvam Associates</t>
+  </si>
+  <si>
+    <t>Anhad Law</t>
+  </si>
+  <si>
+    <t>10s</t>
+  </si>
+  <si>
+    <t>Economic Laws Practice</t>
+  </si>
+  <si>
+    <t>MAS Law</t>
+  </si>
+  <si>
+    <t>09s</t>
+  </si>
+  <si>
+    <t>Arnold Bloch Leibler</t>
+  </si>
+  <si>
+    <t>Vellani &amp; Vellani</t>
+  </si>
+  <si>
+    <t>07s</t>
+  </si>
+  <si>
+    <t>LNT</t>
+  </si>
+  <si>
+    <t>Sok Siphana &amp; Associates</t>
+  </si>
+  <si>
+    <t>Dashnyam</t>
+  </si>
+  <si>
+    <t>05s</t>
+  </si>
+  <si>
+    <t>K1 Chamber</t>
+  </si>
+  <si>
+    <t>Aequitas</t>
+  </si>
+  <si>
+    <t>04s</t>
+  </si>
+  <si>
+    <t>BTG Advaya</t>
+  </si>
+  <si>
+    <t>03s</t>
+  </si>
+  <si>
+    <t>Samvad Partners</t>
+  </si>
+  <si>
+    <t>AOil</t>
+  </si>
+  <si>
+    <t>01s</t>
+  </si>
+  <si>
+    <t>Corrs</t>
+  </si>
+  <si>
+    <t>01min 37s</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Simpson Grierson</t>
+  </si>
+  <si>
+    <t>01min 19s</t>
+  </si>
+  <si>
+    <t>Wenger Vieli AG</t>
+  </si>
+  <si>
+    <t>Minter Ellison RuddWatts</t>
+  </si>
+  <si>
+    <t>Gilbert + Tobin</t>
+  </si>
+  <si>
+    <t>Hicksons</t>
   </si>
   <si>
     <t>01min 04s</t>
   </si>
   <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>Schoenherr</t>
-  </si>
-  <si>
-    <t>Houthoof</t>
-  </si>
-  <si>
-    <t>01min 06s</t>
-  </si>
-  <si>
-    <t>Young List</t>
-  </si>
-  <si>
-    <t>01min 09s</t>
-  </si>
-  <si>
-    <t>Hakun Law</t>
-  </si>
-  <si>
-    <t>01min 43s</t>
-  </si>
-  <si>
-    <t>Nauta Dutilh</t>
-  </si>
-  <si>
-    <t>02min 10s</t>
-  </si>
-  <si>
-    <t>Latham And Watkins</t>
-  </si>
-  <si>
-    <t>02min 29s</t>
-  </si>
-  <si>
-    <t>Guantao Law</t>
-  </si>
-  <si>
-    <t>03min 48s</t>
-  </si>
-  <si>
-    <t>Tahota Law</t>
-  </si>
-  <si>
-    <t>04min 00s</t>
-  </si>
-  <si>
-    <t>Davies Ward Phillips And Vineberg</t>
-  </si>
-  <si>
-    <t>Huiye Law</t>
-  </si>
-  <si>
-    <t>Ashurst</t>
-  </si>
-  <si>
-    <t>Gadens</t>
-  </si>
-  <si>
-    <t>Ronan Daly Jermyn</t>
-  </si>
-  <si>
-    <t>05s</t>
-  </si>
-  <si>
-    <t>Werksmans</t>
-  </si>
-  <si>
-    <t>08s</t>
-  </si>
-  <si>
-    <t>Banki Haddock Fiora</t>
-  </si>
-  <si>
-    <t>Schindler Attorneys</t>
-  </si>
-  <si>
-    <t>10s</t>
-  </si>
-  <si>
-    <t>StewartMcKelvey</t>
-  </si>
-  <si>
-    <t>13s</t>
-  </si>
-  <si>
-    <t>Bennett Jones</t>
-  </si>
-  <si>
-    <t>14s</t>
-  </si>
-  <si>
-    <t>Helmsman</t>
-  </si>
-  <si>
-    <t>17s</t>
-  </si>
-  <si>
-    <t>MBIP</t>
-  </si>
-  <si>
-    <t>18s</t>
-  </si>
-  <si>
-    <t>Hammarskiöld And Co</t>
-  </si>
-  <si>
-    <t>Krogerus</t>
-  </si>
-  <si>
-    <t>Reliance Corporate Advisors</t>
-  </si>
-  <si>
-    <t>21s</t>
-  </si>
-  <si>
-    <t>Paksoy</t>
-  </si>
-  <si>
-    <t>Dillon Eustace</t>
+    <t>Buddle Findlay</t>
+  </si>
+  <si>
+    <t>Moray &amp; Agnew</t>
+  </si>
+  <si>
+    <t>HWL Ebsworth</t>
+  </si>
+  <si>
+    <t>53s</t>
+  </si>
+  <si>
+    <t>Norman Waterhouse</t>
+  </si>
+  <si>
+    <t>52s</t>
+  </si>
+  <si>
+    <t>Tompkins Wake</t>
+  </si>
+  <si>
+    <t>49s</t>
+  </si>
+  <si>
+    <t>Zhong Lun</t>
+  </si>
+  <si>
+    <t>39s</t>
+  </si>
+  <si>
+    <t>Hesketh Henry</t>
+  </si>
+  <si>
+    <t>Baumgartners</t>
+  </si>
+  <si>
+    <t>Mellor Olsson</t>
+  </si>
+  <si>
+    <t>Carter Newell</t>
+  </si>
+  <si>
+    <t>DW Fox Tucker</t>
+  </si>
+  <si>
+    <t>FPA Patent</t>
+  </si>
+  <si>
+    <t>wilson ryan grose</t>
+  </si>
+  <si>
+    <t>Johnson Winter Slattery</t>
+  </si>
+  <si>
+    <t>McCullough Robertson</t>
+  </si>
+  <si>
+    <t>Wilson Harle</t>
+  </si>
+  <si>
+    <t>Anderson Lloyd</t>
+  </si>
+  <si>
+    <t>Greenwood Roche</t>
   </si>
   <si>
     <t>DBHLaw</t>
   </si>
   <si>
-    <t>25s</t>
-  </si>
-  <si>
-    <t>James And Wells</t>
-  </si>
-  <si>
-    <t>Ramdas And Wong</t>
-  </si>
-  <si>
-    <t>MSP</t>
-  </si>
-  <si>
-    <t>28s</t>
-  </si>
-  <si>
-    <t>Carey Olsen</t>
-  </si>
-  <si>
-    <t>Dahl Law</t>
-  </si>
-  <si>
-    <t>29s</t>
-  </si>
-  <si>
-    <t>Santamarina And Steta</t>
-  </si>
-  <si>
-    <t>34s</t>
-  </si>
-  <si>
-    <t>Saba And Co</t>
-  </si>
-  <si>
-    <t>55s</t>
+    <t>Lane Neave</t>
+  </si>
+  <si>
+    <t>Macpherson Kelley</t>
+  </si>
+  <si>
+    <t>Docvit</t>
+  </si>
+  <si>
+    <t>Finlaysons</t>
+  </si>
+  <si>
+    <t>Corcoran</t>
   </si>
 </sst>
 </file>
@@ -1192,13 +1666,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C144"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="1" width="27.6634615384615"/>
-    <col min="2" max="2" customWidth="true" style="1" width="33.3461538461538"/>
-    <col min="3" max="3" customWidth="true" style="1" width="51.1442307692308"/>
-    <col min="4" max="8" customWidth="true" width="8.88461538461539"/>
+    <col min="1" max="1" width="27.6634615384615" style="1" customWidth="1"/>
+    <col min="2" max="2" width="33.3461538461538" style="1" customWidth="1"/>
+    <col min="3" max="3" width="51.1442307692308" style="1" customWidth="1"/>
+    <col min="4" max="8" width="8.88461538461539" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="23.2" spans="1:3">
@@ -1212,9 +1686,1560 @@
         <v>2</v>
       </c>
     </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
+      <c r="A44" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
+      <c r="A45" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
+      <c r="A46" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3">
+      <c r="A47" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
+      <c r="A48" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="A49" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3">
+      <c r="A50" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3">
+      <c r="A51" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3">
+      <c r="A52" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3">
+      <c r="A53" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
+      <c r="A55" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3">
+      <c r="A56" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3">
+      <c r="A57" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3">
+      <c r="A58" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3">
+      <c r="A59" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3">
+      <c r="A60" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="A63" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3">
+      <c r="A64" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3">
+      <c r="A65" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3">
+      <c r="A66" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3">
+      <c r="A67" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3">
+      <c r="A68" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3">
+      <c r="A69" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3">
+      <c r="A70" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3">
+      <c r="A71" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3">
+      <c r="A72" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3">
+      <c r="A73" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3">
+      <c r="A74" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3">
+      <c r="A75" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3">
+      <c r="A76" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3">
+      <c r="A77" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3">
+      <c r="A78" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3">
+      <c r="A79" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3">
+      <c r="A80" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3">
+      <c r="A81" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3">
+      <c r="A82" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3">
+      <c r="A83" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3">
+      <c r="A84" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3">
+      <c r="A85" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3">
+      <c r="A86" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3">
+      <c r="A87" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3">
+      <c r="A88" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3">
+      <c r="A89" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3">
+      <c r="A90" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3">
+      <c r="A91" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3">
+      <c r="A92" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3">
+      <c r="A93" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3">
+      <c r="A94" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C94" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3">
+      <c r="A95" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C95" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3">
+      <c r="A96" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C96" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3">
+      <c r="A97" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C97" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3">
+      <c r="A98" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C98" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3">
+      <c r="A99" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C99" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3">
+      <c r="A100" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3">
+      <c r="A101" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C101" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3">
+      <c r="A102" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="C102" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3">
+      <c r="A103" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="C103" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3">
+      <c r="A104" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3">
+      <c r="A105" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C105" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3">
+      <c r="A106" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C106" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3">
+      <c r="A107" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C107" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3">
+      <c r="A108" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C108" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3">
+      <c r="A109" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="C109" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3">
+      <c r="A110" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3">
+      <c r="A111" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="C111" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3">
+      <c r="A112" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="C112" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3">
+      <c r="A113" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="C113" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3">
+      <c r="A114" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="C114" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3">
+      <c r="A115" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="C115" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3">
+      <c r="A116" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="C116" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3">
+      <c r="A117" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C117" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3">
+      <c r="A118" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="B118" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C118" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3">
+      <c r="A119" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B119" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C119" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3">
+      <c r="A120" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="B120" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="C120" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3">
+      <c r="A121" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="B121" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C121" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3">
+      <c r="A122" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C122" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3">
+      <c r="A123" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="B123" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="C123" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3">
+      <c r="A124" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="B124" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="C124" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3">
+      <c r="A125" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B125" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="C125" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3">
+      <c r="A126" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="B126" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="C126" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3">
+      <c r="A127" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="B127" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C127" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3">
+      <c r="A128" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="B128" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C128" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3">
+      <c r="A129" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="B129" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C129" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3">
+      <c r="A130" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B130" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C130" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3">
+      <c r="A131" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="B131" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C131" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3">
+      <c r="A132" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="B132" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C132" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3">
+      <c r="A133" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="B133" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C133" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3">
+      <c r="A134" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="B134" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C134" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3">
+      <c r="A135" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="B135" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C135" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3">
+      <c r="A136" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="B136" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C136" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3">
+      <c r="A137" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="B137" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C137" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3">
+      <c r="A138" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B138" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C138" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3">
+      <c r="A139" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="B139" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C139" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3">
+      <c r="A140" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="B140" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C140" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3">
+      <c r="A141" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="B141" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C141" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3">
+      <c r="A142" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="B142" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C142" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3">
+      <c r="A143" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="B143" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C143" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3">
+      <c r="A144" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="B144" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C144" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState ref="A2:C35">
-    <sortCondition ref="B2"/>
+  <sortState ref="A2:C350">
+    <sortCondition ref="C2"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
@@ -1227,8 +3252,8 @@
   <dimension ref="D2:F35"/>
   <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelCol="5"/>
   <cols>
-    <col min="4" max="4" customWidth="true" width="36.0769230769231"/>
-    <col min="5" max="6" customWidth="true" width="15.875"/>
+    <col min="4" max="4" width="36.0769230769231" customWidth="1"/>
+    <col min="5" max="6" width="15.875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="4:6">

</xml_diff>